<commit_message>
add kor pcba plat
</commit_message>
<xml_diff>
--- a/data/premium/TASA-EFX_KOR_Platinum_Model_2024_v3.0-test.xlsx
+++ b/data/premium/TASA-EFX_KOR_Platinum_Model_2024_v3.0-test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EllieS\Documents\GitHub\TASA_EFX_dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EllieS\Documents\GitHub\Ellie_dashboard_attempt\data\premium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F46F584-1950-4D8A-88ED-18B90EA487A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99DBC0C1-7018-456E-A4A4-ED141CEAE0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51720" yWindow="7725" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legal" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2446" uniqueCount="1446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2551" uniqueCount="1446">
   <si>
     <t>By using these data, you agree to comply with the full data license, as signed and agreed to by you or your company. Key clauses are summarized below. </t>
   </si>
@@ -4494,7 +4494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4533,11 +4533,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="###0"/>
       <border>
@@ -5013,7 +5035,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AK23"/>
+  <dimension ref="A1:AK44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="45.68359375" customWidth="1"/>
@@ -7555,11 +7577,2389 @@
         <v>43</v>
       </c>
     </row>
+    <row r="24" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" t="s">
+        <v>188</v>
+      </c>
+      <c r="B24" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C24" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D24" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E24" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F24" t="s">
+        <v>188</v>
+      </c>
+      <c r="G24" s="14">
+        <v>115.6367781318685</v>
+      </c>
+      <c r="H24" s="14">
+        <v>3.8723710837708918</v>
+      </c>
+      <c r="I24" s="14">
+        <v>20.457593305325311</v>
+      </c>
+      <c r="J24" s="14">
+        <v>91.306813742772306</v>
+      </c>
+      <c r="K24" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L24" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M24" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N24" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O24" t="s">
+        <v>188</v>
+      </c>
+      <c r="P24" s="14">
+        <v>115.24479558484209</v>
+      </c>
+      <c r="Q24" s="14">
+        <v>4.187498421574535</v>
+      </c>
+      <c r="R24" s="14">
+        <v>18.802387447074789</v>
+      </c>
+      <c r="S24" s="14">
+        <v>92.254909716192756</v>
+      </c>
+      <c r="T24" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U24" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V24" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W24" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X24" t="s">
+        <v>188</v>
+      </c>
+      <c r="Y24" s="14">
+        <v>117.8816565777712</v>
+      </c>
+      <c r="Z24" s="14">
+        <v>4.346034855990176</v>
+      </c>
+      <c r="AA24" s="14">
+        <v>18.929562392723831</v>
+      </c>
+      <c r="AB24" s="14">
+        <v>94.606059329057175</v>
+      </c>
+      <c r="AC24" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD24" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE24" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF24" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>188</v>
+      </c>
+      <c r="AH24" s="14">
+        <v>119.9017036758714</v>
+      </c>
+      <c r="AI24" s="14">
+        <v>4.4205095058547492</v>
+      </c>
+      <c r="AJ24" s="14">
+        <v>19.25394371454977</v>
+      </c>
+      <c r="AK24" s="14">
+        <v>96.227250455466887</v>
+      </c>
+    </row>
+    <row r="25" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" t="s">
+        <v>188</v>
+      </c>
+      <c r="B25" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C25" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D25" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E25" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F25" t="s">
+        <v>115</v>
+      </c>
+      <c r="G25" s="14">
+        <v>35.914985459227722</v>
+      </c>
+      <c r="H25" s="14">
+        <v>6.6136239293297852</v>
+      </c>
+      <c r="I25" s="14">
+        <v>4.9506844991757397</v>
+      </c>
+      <c r="J25" s="14">
+        <v>24.350677030722199</v>
+      </c>
+      <c r="K25" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L25" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M25" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N25" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O25" t="s">
+        <v>115</v>
+      </c>
+      <c r="P25" s="14">
+        <v>36.784175251509957</v>
+      </c>
+      <c r="Q25" s="14">
+        <v>7.1518300198614417</v>
+      </c>
+      <c r="R25" s="14">
+        <v>4.5501289761928554</v>
+      </c>
+      <c r="S25" s="14">
+        <v>25.082216255455659</v>
+      </c>
+      <c r="T25" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U25" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V25" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W25" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X25" t="s">
+        <v>115</v>
+      </c>
+      <c r="Y25" s="14">
+        <v>37.815168607372698</v>
+      </c>
+      <c r="Z25" s="14">
+        <v>7.4225944516887976</v>
+      </c>
+      <c r="AA25" s="14">
+        <v>4.5809049830628492</v>
+      </c>
+      <c r="AB25" s="14">
+        <v>25.811669172621041</v>
+      </c>
+      <c r="AC25" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD25" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE25" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF25" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH25" s="14">
+        <v>38.463178007877659</v>
+      </c>
+      <c r="AI25" s="14">
+        <v>7.5497897322591614</v>
+      </c>
+      <c r="AJ25" s="14">
+        <v>4.6594044212820931</v>
+      </c>
+      <c r="AK25" s="14">
+        <v>26.253983854336401</v>
+      </c>
+    </row>
+    <row r="26" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" t="s">
+        <v>188</v>
+      </c>
+      <c r="B26" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C26" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D26" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E26" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F26" t="s">
+        <v>167</v>
+      </c>
+      <c r="G26" s="14">
+        <v>32.526099180771887</v>
+      </c>
+      <c r="H26" s="14">
+        <v>0.61935491475764515</v>
+      </c>
+      <c r="I26" s="14">
+        <v>2.3299192612181741</v>
+      </c>
+      <c r="J26" s="14">
+        <v>29.576825004796071</v>
+      </c>
+      <c r="K26" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L26" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M26" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N26" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O26" t="s">
+        <v>167</v>
+      </c>
+      <c r="P26" s="14">
+        <v>32.588709845907658</v>
+      </c>
+      <c r="Q26" s="14">
+        <v>0.6697570227222357</v>
+      </c>
+      <c r="R26" s="14">
+        <v>2.141407545648232</v>
+      </c>
+      <c r="S26" s="14">
+        <v>29.77754527753719</v>
+      </c>
+      <c r="T26" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U26" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V26" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W26" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X26" t="s">
+        <v>167</v>
+      </c>
+      <c r="Y26" s="14">
+        <v>33.367388717251423</v>
+      </c>
+      <c r="Z26" s="14">
+        <v>0.69511366280122922</v>
+      </c>
+      <c r="AA26" s="14">
+        <v>2.1558915248235802</v>
+      </c>
+      <c r="AB26" s="14">
+        <v>30.516383529626619</v>
+      </c>
+      <c r="AC26" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD26" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE26" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF26" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG26" t="s">
+        <v>167</v>
+      </c>
+      <c r="AH26" s="14">
+        <v>33.939179941656192</v>
+      </c>
+      <c r="AI26" s="14">
+        <v>0.70702528992079761</v>
+      </c>
+      <c r="AJ26" s="14">
+        <v>2.1928353763520452</v>
+      </c>
+      <c r="AK26" s="14">
+        <v>31.039319275383338</v>
+      </c>
+    </row>
+    <row r="27" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" t="s">
+        <v>188</v>
+      </c>
+      <c r="B27" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C27" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D27" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E27" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F27" t="s">
+        <v>262</v>
+      </c>
+      <c r="G27" s="14">
+        <v>22.12444242749406</v>
+      </c>
+      <c r="H27" s="14">
+        <v>1.8119866900241399</v>
+      </c>
+      <c r="I27" s="14">
+        <v>3.7504219498165989</v>
+      </c>
+      <c r="J27" s="14">
+        <v>16.56203378765332</v>
+      </c>
+      <c r="K27" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L27" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M27" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N27" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O27" t="s">
+        <v>262</v>
+      </c>
+      <c r="P27" s="14">
+        <v>22.219564342725992</v>
+      </c>
+      <c r="Q27" s="14">
+        <v>1.95944325588789</v>
+      </c>
+      <c r="R27" s="14">
+        <v>3.4469786126850601</v>
+      </c>
+      <c r="S27" s="14">
+        <v>16.81314247415304</v>
+      </c>
+      <c r="T27" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U27" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V27" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W27" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X27" t="s">
+        <v>262</v>
+      </c>
+      <c r="Y27" s="14">
+        <v>22.760466656317622</v>
+      </c>
+      <c r="Z27" s="14">
+        <v>2.0336267219944721</v>
+      </c>
+      <c r="AA27" s="14">
+        <v>3.470293168826164</v>
+      </c>
+      <c r="AB27" s="14">
+        <v>17.256546765496982</v>
+      </c>
+      <c r="AC27" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD27" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE27" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF27" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG27" t="s">
+        <v>262</v>
+      </c>
+      <c r="AH27" s="14">
+        <v>23.150495232054229</v>
+      </c>
+      <c r="AI27" s="14">
+        <v>2.068475415825592</v>
+      </c>
+      <c r="AJ27" s="14">
+        <v>3.5297609083265802</v>
+      </c>
+      <c r="AK27" s="14">
+        <v>17.552258907902061</v>
+      </c>
+    </row>
+    <row r="28" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" t="s">
+        <v>188</v>
+      </c>
+      <c r="B28" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C28" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D28" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E28" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F28" t="s">
+        <v>128</v>
+      </c>
+      <c r="G28" s="14">
+        <v>16.016182927977951</v>
+      </c>
+      <c r="H28" s="14">
+        <v>1.1284012295670649</v>
+      </c>
+      <c r="I28" s="14">
+        <v>2.4232337856164521</v>
+      </c>
+      <c r="J28" s="14">
+        <v>12.464547912794441</v>
+      </c>
+      <c r="K28" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L28" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M28" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N28" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O28" t="s">
+        <v>128</v>
+      </c>
+      <c r="P28" s="14">
+        <v>16.15331379439969</v>
+      </c>
+      <c r="Q28" s="14">
+        <v>1.2202287088440651</v>
+      </c>
+      <c r="R28" s="14">
+        <v>2.2271720740553529</v>
+      </c>
+      <c r="S28" s="14">
+        <v>12.705913011500281</v>
+      </c>
+      <c r="T28" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U28" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V28" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W28" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X28" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y28" s="14">
+        <v>16.559487874822459</v>
+      </c>
+      <c r="Z28" s="14">
+        <v>1.266425910417935</v>
+      </c>
+      <c r="AA28" s="14">
+        <v>2.2422361444169678</v>
+      </c>
+      <c r="AB28" s="14">
+        <v>13.05082581998755</v>
+      </c>
+      <c r="AC28" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD28" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE28" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF28" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AH28" s="14">
+        <v>16.84325505623708</v>
+      </c>
+      <c r="AI28" s="14">
+        <v>1.2881276752180499</v>
+      </c>
+      <c r="AJ28" s="14">
+        <v>2.2806596171461342</v>
+      </c>
+      <c r="AK28" s="14">
+        <v>13.274467763872901</v>
+      </c>
+    </row>
+    <row r="29" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" t="s">
+        <v>188</v>
+      </c>
+      <c r="B29" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C29" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D29" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E29" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F29" t="s">
+        <v>177</v>
+      </c>
+      <c r="G29" s="14">
+        <v>14.725922171802971</v>
+      </c>
+      <c r="H29" s="14">
+        <v>2.462896543760547</v>
+      </c>
+      <c r="I29" s="14">
+        <v>3.2701248699144858</v>
+      </c>
+      <c r="J29" s="14">
+        <v>8.9929007581279414</v>
+      </c>
+      <c r="K29" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L29" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M29" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N29" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O29" t="s">
+        <v>177</v>
+      </c>
+      <c r="P29" s="14">
+        <v>14.783236825338619</v>
+      </c>
+      <c r="Q29" s="14">
+        <v>2.6633231078297288</v>
+      </c>
+      <c r="R29" s="14">
+        <v>3.005541946541765</v>
+      </c>
+      <c r="S29" s="14">
+        <v>9.114371770967125</v>
+      </c>
+      <c r="T29" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U29" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V29" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W29" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X29" t="s">
+        <v>177</v>
+      </c>
+      <c r="Y29" s="14">
+        <v>15.141975425518821</v>
+      </c>
+      <c r="Z29" s="14">
+        <v>2.7641550859474302</v>
+      </c>
+      <c r="AA29" s="14">
+        <v>3.0258707284463648</v>
+      </c>
+      <c r="AB29" s="14">
+        <v>9.3519496111250202</v>
+      </c>
+      <c r="AC29" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD29" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE29" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF29" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG29" t="s">
+        <v>177</v>
+      </c>
+      <c r="AH29" s="14">
+        <v>15.40145178855791</v>
+      </c>
+      <c r="AI29" s="14">
+        <v>2.811522281337862</v>
+      </c>
+      <c r="AJ29" s="14">
+        <v>3.077722743099653</v>
+      </c>
+      <c r="AK29" s="14">
+        <v>9.512206764120398</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" t="s">
+        <v>188</v>
+      </c>
+      <c r="B30" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C30" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D30" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E30" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F30" t="s">
+        <v>178</v>
+      </c>
+      <c r="G30" s="14">
+        <v>12.733258666732629</v>
+      </c>
+      <c r="H30" s="14">
+        <v>1.160142255602058</v>
+      </c>
+      <c r="I30" s="14">
+        <v>1.260828033247257</v>
+      </c>
+      <c r="J30" s="14">
+        <v>10.312288377883309</v>
+      </c>
+      <c r="K30" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L30" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M30" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N30" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O30" t="s">
+        <v>178</v>
+      </c>
+      <c r="P30" s="14">
+        <v>13.107302020376681</v>
+      </c>
+      <c r="Q30" s="14">
+        <v>1.254552768585586</v>
+      </c>
+      <c r="R30" s="14">
+        <v>1.1588155474318269</v>
+      </c>
+      <c r="S30" s="14">
+        <v>10.69393370435926</v>
+      </c>
+      <c r="T30" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U30" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V30" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W30" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X30" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y30" s="14">
+        <v>13.486925659812661</v>
+      </c>
+      <c r="Z30" s="14">
+        <v>1.3020494605707369</v>
+      </c>
+      <c r="AA30" s="14">
+        <v>1.1666535044294011</v>
+      </c>
+      <c r="AB30" s="14">
+        <v>11.018222694812531</v>
+      </c>
+      <c r="AC30" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD30" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE30" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF30" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG30" t="s">
+        <v>178</v>
+      </c>
+      <c r="AH30" s="14">
+        <v>13.7180407105536</v>
+      </c>
+      <c r="AI30" s="14">
+        <v>1.324361678694967</v>
+      </c>
+      <c r="AJ30" s="14">
+        <v>1.186645546402074</v>
+      </c>
+      <c r="AK30" s="14">
+        <v>11.207033485456559</v>
+      </c>
+    </row>
+    <row r="31" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C31" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D31" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E31" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F31" t="s">
+        <v>288</v>
+      </c>
+      <c r="G31" s="14">
+        <v>9.9769304277994664</v>
+      </c>
+      <c r="H31" s="14">
+        <v>1.4243067803255109</v>
+      </c>
+      <c r="I31" s="14">
+        <v>2.1729476335415399</v>
+      </c>
+      <c r="J31" s="14">
+        <v>6.3796760139324151</v>
+      </c>
+      <c r="K31" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L31" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M31" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N31" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O31" t="s">
+        <v>288</v>
+      </c>
+      <c r="P31" s="14">
+        <v>9.9527521115008764</v>
+      </c>
+      <c r="Q31" s="14">
+        <v>1.5402145779487131</v>
+      </c>
+      <c r="R31" s="14">
+        <v>1.9971363541290541</v>
+      </c>
+      <c r="S31" s="14">
+        <v>6.4154011794231094</v>
+      </c>
+      <c r="T31" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U31" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V31" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W31" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X31" t="s">
+        <v>288</v>
+      </c>
+      <c r="Y31" s="14">
+        <v>10.182318558089531</v>
+      </c>
+      <c r="Z31" s="14">
+        <v>1.598526272148987</v>
+      </c>
+      <c r="AA31" s="14">
+        <v>2.010644516749625</v>
+      </c>
+      <c r="AB31" s="14">
+        <v>6.573147769190915</v>
+      </c>
+      <c r="AC31" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD31" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE31" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF31" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG31" t="s">
+        <v>288</v>
+      </c>
+      <c r="AH31" s="14">
+        <v>10.35680510376876</v>
+      </c>
+      <c r="AI31" s="14">
+        <v>1.625918984900365</v>
+      </c>
+      <c r="AJ31" s="14">
+        <v>2.0450993822417098</v>
+      </c>
+      <c r="AK31" s="14">
+        <v>6.6857867366266843</v>
+      </c>
+    </row>
+    <row r="32" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" t="s">
+        <v>188</v>
+      </c>
+      <c r="B32" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C32" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D32" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E32" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F32" t="s">
+        <v>127</v>
+      </c>
+      <c r="G32" s="14">
+        <v>8.8453747795196165</v>
+      </c>
+      <c r="H32" s="14">
+        <v>0.93739417071827735</v>
+      </c>
+      <c r="I32" s="14">
+        <v>0.93395478034051616</v>
+      </c>
+      <c r="J32" s="14">
+        <v>6.9740258284608228</v>
+      </c>
+      <c r="K32" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L32" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M32" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N32" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O32" t="s">
+        <v>127</v>
+      </c>
+      <c r="P32" s="14">
+        <v>8.9537440355774134</v>
+      </c>
+      <c r="Q32" s="14">
+        <v>1.013677802400458</v>
+      </c>
+      <c r="R32" s="14">
+        <v>0.85838932155518122</v>
+      </c>
+      <c r="S32" s="14">
+        <v>7.0816769116217744</v>
+      </c>
+      <c r="T32" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U32" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V32" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W32" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X32" t="s">
+        <v>127</v>
+      </c>
+      <c r="Y32" s="14">
+        <v>9.1850475262098659</v>
+      </c>
+      <c r="Z32" s="14">
+        <v>1.052055097926321</v>
+      </c>
+      <c r="AA32" s="14">
+        <v>0.86419526591314011</v>
+      </c>
+      <c r="AB32" s="14">
+        <v>7.2687971623704053</v>
+      </c>
+      <c r="AC32" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD32" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE32" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF32" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG32" t="s">
+        <v>127</v>
+      </c>
+      <c r="AH32" s="14">
+        <v>9.3424446068064704</v>
+      </c>
+      <c r="AI32" s="14">
+        <v>1.070083355327043</v>
+      </c>
+      <c r="AJ32" s="14">
+        <v>0.87900431415507807</v>
+      </c>
+      <c r="AK32" s="14">
+        <v>7.3933569373243504</v>
+      </c>
+    </row>
+    <row r="33" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C33" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D33" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E33" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F33" t="s">
+        <v>335</v>
+      </c>
+      <c r="G33" s="14">
+        <v>8.6741189011365609</v>
+      </c>
+      <c r="H33" s="14">
+        <v>1.052998146749927</v>
+      </c>
+      <c r="I33" s="14">
+        <v>4.6614934655072329</v>
+      </c>
+      <c r="J33" s="14">
+        <v>2.9596272888794002</v>
+      </c>
+      <c r="K33" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L33" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M33" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N33" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O33" t="s">
+        <v>335</v>
+      </c>
+      <c r="P33" s="14">
+        <v>8.3812621205283637</v>
+      </c>
+      <c r="Q33" s="14">
+        <v>1.138689444282895</v>
+      </c>
+      <c r="R33" s="14">
+        <v>4.2843361343809159</v>
+      </c>
+      <c r="S33" s="14">
+        <v>2.9582365418645522</v>
+      </c>
+      <c r="T33" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U33" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V33" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W33" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X33" t="s">
+        <v>335</v>
+      </c>
+      <c r="Y33" s="14">
+        <v>8.5226878306630542</v>
+      </c>
+      <c r="Z33" s="14">
+        <v>1.181799613226066</v>
+      </c>
+      <c r="AA33" s="14">
+        <v>4.3133143807108461</v>
+      </c>
+      <c r="AB33" s="14">
+        <v>3.0275738367261402</v>
+      </c>
+      <c r="AC33" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD33" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE33" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF33" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG33" t="s">
+        <v>335</v>
+      </c>
+      <c r="AH33" s="14">
+        <v>8.6687345636336453</v>
+      </c>
+      <c r="AI33" s="14">
+        <v>1.2020512023921739</v>
+      </c>
+      <c r="AJ33" s="14">
+        <v>4.387228325008028</v>
+      </c>
+      <c r="AK33" s="14">
+        <v>3.0794550362334432</v>
+      </c>
+    </row>
+    <row r="34" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" t="s">
+        <v>188</v>
+      </c>
+      <c r="B34" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C34" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D34" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E34" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F34" t="s">
+        <v>169</v>
+      </c>
+      <c r="G34" s="14">
+        <v>7.2300521184473467</v>
+      </c>
+      <c r="H34" s="14">
+        <v>2.2463193029968589</v>
+      </c>
+      <c r="I34" s="14">
+        <v>0.40457415074079289</v>
+      </c>
+      <c r="J34" s="14">
+        <v>4.5791586647096949</v>
+      </c>
+      <c r="K34" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L34" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M34" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N34" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O34" t="s">
+        <v>271</v>
+      </c>
+      <c r="P34" s="14">
+        <v>7.5567330610634764</v>
+      </c>
+      <c r="Q34" s="14">
+        <v>6.3425308165652403</v>
+      </c>
+      <c r="R34" s="14">
+        <v>0.34573481265762018</v>
+      </c>
+      <c r="S34" s="14">
+        <v>0.86846743184061537</v>
+      </c>
+      <c r="T34" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U34" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V34" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W34" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X34" t="s">
+        <v>271</v>
+      </c>
+      <c r="Y34" s="14">
+        <v>7.8250843651925246</v>
+      </c>
+      <c r="Z34" s="14">
+        <v>6.5826556165291059</v>
+      </c>
+      <c r="AA34" s="14">
+        <v>0.34807328196809889</v>
+      </c>
+      <c r="AB34" s="14">
+        <v>0.89435546669531985</v>
+      </c>
+      <c r="AC34" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD34" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE34" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF34" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG34" t="s">
+        <v>271</v>
+      </c>
+      <c r="AH34" s="14">
+        <v>7.9591768052140814</v>
+      </c>
+      <c r="AI34" s="14">
+        <v>6.6954575126170681</v>
+      </c>
+      <c r="AJ34" s="14">
+        <v>0.35403794554323281</v>
+      </c>
+      <c r="AK34" s="14">
+        <v>0.90968134705377934</v>
+      </c>
+    </row>
+    <row r="35" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" t="s">
+        <v>188</v>
+      </c>
+      <c r="B35" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C35" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D35" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E35" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F35" t="s">
+        <v>162</v>
+      </c>
+      <c r="G35" s="14">
+        <v>7.1427015990240408</v>
+      </c>
+      <c r="H35" s="14">
+        <v>2.7114566102660742</v>
+      </c>
+      <c r="I35" s="14">
+        <v>0.43262662042217598</v>
+      </c>
+      <c r="J35" s="14">
+        <v>3.9986183683357899</v>
+      </c>
+      <c r="K35" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L35" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M35" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N35" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O35" t="s">
+        <v>162</v>
+      </c>
+      <c r="P35" s="14">
+        <v>7.5171563874339986</v>
+      </c>
+      <c r="Q35" s="14">
+        <v>2.9321105932338352</v>
+      </c>
+      <c r="R35" s="14">
+        <v>0.39762318155864629</v>
+      </c>
+      <c r="S35" s="14">
+        <v>4.1874226126415168</v>
+      </c>
+      <c r="T35" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U35" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V35" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W35" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X35" t="s">
+        <v>162</v>
+      </c>
+      <c r="Y35" s="14">
+        <v>7.7653320057553961</v>
+      </c>
+      <c r="Z35" s="14">
+        <v>3.0431187207518491</v>
+      </c>
+      <c r="AA35" s="14">
+        <v>0.40031261164542958</v>
+      </c>
+      <c r="AB35" s="14">
+        <v>4.321900673358118</v>
+      </c>
+      <c r="AC35" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD35" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE35" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF35" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG35" t="s">
+        <v>162</v>
+      </c>
+      <c r="AH35" s="14">
+        <v>7.8984005156440578</v>
+      </c>
+      <c r="AI35" s="14">
+        <v>3.0952663009563541</v>
+      </c>
+      <c r="AJ35" s="14">
+        <v>0.40717246035271148</v>
+      </c>
+      <c r="AK35" s="14">
+        <v>4.3959617543349916</v>
+      </c>
+    </row>
+    <row r="36" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" t="s">
+        <v>188</v>
+      </c>
+      <c r="B36" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C36" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D36" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E36" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F36" t="s">
+        <v>271</v>
+      </c>
+      <c r="G36" s="14">
+        <v>7.0812237693020537</v>
+      </c>
+      <c r="H36" s="14">
+        <v>5.8652279856282359</v>
+      </c>
+      <c r="I36" s="14">
+        <v>0.37617043094933178</v>
+      </c>
+      <c r="J36" s="14">
+        <v>0.83982535272448544</v>
+      </c>
+      <c r="K36" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L36" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M36" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N36" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O36" t="s">
+        <v>169</v>
+      </c>
+      <c r="P36" s="14">
+        <v>7.4194822381528729</v>
+      </c>
+      <c r="Q36" s="14">
+        <v>2.4291211591456778</v>
+      </c>
+      <c r="R36" s="14">
+        <v>0.37184041249463412</v>
+      </c>
+      <c r="S36" s="14">
+        <v>4.6185206665125609</v>
+      </c>
+      <c r="T36" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U36" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V36" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W36" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X36" t="s">
+        <v>169</v>
+      </c>
+      <c r="Y36" s="14">
+        <v>7.6301242126534117</v>
+      </c>
+      <c r="Z36" s="14">
+        <v>2.5210863776518959</v>
+      </c>
+      <c r="AA36" s="14">
+        <v>0.37435545396914</v>
+      </c>
+      <c r="AB36" s="14">
+        <v>4.7346823810323757</v>
+      </c>
+      <c r="AC36" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD36" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE36" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF36" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG36" t="s">
+        <v>169</v>
+      </c>
+      <c r="AH36" s="14">
+        <v>7.7608757707955052</v>
+      </c>
+      <c r="AI36" s="14">
+        <v>2.564288291919838</v>
+      </c>
+      <c r="AJ36" s="14">
+        <v>0.3807704948703462</v>
+      </c>
+      <c r="AK36" s="14">
+        <v>4.8158169840053224</v>
+      </c>
+    </row>
+    <row r="37" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" t="s">
+        <v>188</v>
+      </c>
+      <c r="B37" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C37" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D37" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E37" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F37" t="s">
+        <v>65</v>
+      </c>
+      <c r="G37" s="14">
+        <v>6.4704374711157246</v>
+      </c>
+      <c r="H37" s="14">
+        <v>0.55633925943767482</v>
+      </c>
+      <c r="I37" s="14">
+        <v>1.1324166462408189</v>
+      </c>
+      <c r="J37" s="14">
+        <v>4.781681565437232</v>
+      </c>
+      <c r="K37" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L37" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M37" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N37" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O37" t="s">
+        <v>110</v>
+      </c>
+      <c r="P37" s="14">
+        <v>6.6293186939445539</v>
+      </c>
+      <c r="Q37" s="14">
+        <v>1.138744421045087</v>
+      </c>
+      <c r="R37" s="14">
+        <v>0.55338079633067117</v>
+      </c>
+      <c r="S37" s="14">
+        <v>4.9371934765687948</v>
+      </c>
+      <c r="T37" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U37" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V37" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W37" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X37" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y37" s="14">
+        <v>6.8257953504941602</v>
+      </c>
+      <c r="Z37" s="14">
+        <v>1.1818566713788581</v>
+      </c>
+      <c r="AA37" s="14">
+        <v>0.55712373444928376</v>
+      </c>
+      <c r="AB37" s="14">
+        <v>5.0868149446660178</v>
+      </c>
+      <c r="AC37" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD37" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE37" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF37" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG37" t="s">
+        <v>110</v>
+      </c>
+      <c r="AH37" s="14">
+        <v>6.9427637448167738</v>
+      </c>
+      <c r="AI37" s="14">
+        <v>1.2021092383065559</v>
+      </c>
+      <c r="AJ37" s="14">
+        <v>0.5666707345146802</v>
+      </c>
+      <c r="AK37" s="14">
+        <v>5.1739837719955357</v>
+      </c>
+    </row>
+    <row r="38" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38" t="s">
+        <v>188</v>
+      </c>
+      <c r="B38" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C38" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D38" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E38" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F38" t="s">
+        <v>110</v>
+      </c>
+      <c r="G38" s="14">
+        <v>6.4166480705614504</v>
+      </c>
+      <c r="H38" s="14">
+        <v>1.053048986273375</v>
+      </c>
+      <c r="I38" s="14">
+        <v>0.60209584055088639</v>
+      </c>
+      <c r="J38" s="14">
+        <v>4.7615032437371889</v>
+      </c>
+      <c r="K38" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L38" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M38" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N38" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O38" t="s">
+        <v>65</v>
+      </c>
+      <c r="P38" s="14">
+        <v>6.4484621428672639</v>
+      </c>
+      <c r="Q38" s="14">
+        <v>0.60161325460745596</v>
+      </c>
+      <c r="R38" s="14">
+        <v>1.0407938126619389</v>
+      </c>
+      <c r="S38" s="14">
+        <v>4.806055075597869</v>
+      </c>
+      <c r="T38" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U38" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V38" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W38" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X38" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y38" s="14">
+        <v>6.6181859344920069</v>
+      </c>
+      <c r="Z38" s="14">
+        <v>0.1039968713338877</v>
+      </c>
+      <c r="AA38" s="14">
+        <v>7.030347003135301E-2</v>
+      </c>
+      <c r="AB38" s="14">
+        <v>6.4438855931267662</v>
+      </c>
+      <c r="AC38" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD38" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE38" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF38" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG38" t="s">
+        <v>163</v>
+      </c>
+      <c r="AH38" s="14">
+        <v>6.7315966862559016</v>
+      </c>
+      <c r="AI38" s="14">
+        <v>0.1057789855681827</v>
+      </c>
+      <c r="AJ38" s="14">
+        <v>7.1508206414825165E-2</v>
+      </c>
+      <c r="AK38" s="14">
+        <v>6.5543094942728928</v>
+      </c>
+    </row>
+    <row r="39" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" t="s">
+        <v>188</v>
+      </c>
+      <c r="B39" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C39" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D39" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E39" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F39" t="s">
+        <v>163</v>
+      </c>
+      <c r="G39" s="14">
+        <v>6.0890116820300788</v>
+      </c>
+      <c r="H39" s="14">
+        <v>9.2662505180077834E-2</v>
+      </c>
+      <c r="I39" s="14">
+        <v>7.5978502197566827E-2</v>
+      </c>
+      <c r="J39" s="14">
+        <v>5.9203706746524336</v>
+      </c>
+      <c r="K39" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L39" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M39" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N39" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O39" t="s">
+        <v>163</v>
+      </c>
+      <c r="P39" s="14">
+        <v>6.4069041684935932</v>
+      </c>
+      <c r="Q39" s="14">
+        <v>0.1002032309886124</v>
+      </c>
+      <c r="R39" s="14">
+        <v>6.983114849561517E-2</v>
+      </c>
+      <c r="S39" s="14">
+        <v>6.236869789009365</v>
+      </c>
+      <c r="T39" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U39" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V39" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W39" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X39" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y39" s="14">
+        <v>6.5959982909120107</v>
+      </c>
+      <c r="Z39" s="14">
+        <v>0.62439000833499381</v>
+      </c>
+      <c r="AA39" s="14">
+        <v>1.047833498283232</v>
+      </c>
+      <c r="AB39" s="14">
+        <v>4.9237747842937836</v>
+      </c>
+      <c r="AC39" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD39" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE39" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF39" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG39" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH39" s="14">
+        <v>6.7090288301277559</v>
+      </c>
+      <c r="AI39" s="14">
+        <v>0.63508969869426313</v>
+      </c>
+      <c r="AJ39" s="14">
+        <v>1.0657894133844319</v>
+      </c>
+      <c r="AK39" s="14">
+        <v>5.0081497180490606</v>
+      </c>
+    </row>
+    <row r="40" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40" t="s">
+        <v>188</v>
+      </c>
+      <c r="B40" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C40" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D40" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E40" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F40" t="s">
+        <v>1390</v>
+      </c>
+      <c r="G40" s="14">
+        <v>5.8884483968019907</v>
+      </c>
+      <c r="H40" s="14">
+        <v>1.2273498912238481</v>
+      </c>
+      <c r="I40" s="14">
+        <v>2.231926860305276</v>
+      </c>
+      <c r="J40" s="14">
+        <v>2.429171645272866</v>
+      </c>
+      <c r="K40" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L40" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M40" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N40" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O40" t="s">
+        <v>294</v>
+      </c>
+      <c r="P40" s="14">
+        <v>6.137752378059373</v>
+      </c>
+      <c r="Q40" s="14">
+        <v>4.6059068750954486</v>
+      </c>
+      <c r="R40" s="14">
+        <v>2.8933133955461331E-2</v>
+      </c>
+      <c r="S40" s="14">
+        <v>1.5029123690084609</v>
+      </c>
+      <c r="T40" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U40" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V40" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W40" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X40" t="s">
+        <v>294</v>
+      </c>
+      <c r="Y40" s="14">
+        <v>6.3509922420448373</v>
+      </c>
+      <c r="Z40" s="14">
+        <v>4.7802840281627841</v>
+      </c>
+      <c r="AA40" s="14">
+        <v>2.9128830898128819E-2</v>
+      </c>
+      <c r="AB40" s="14">
+        <v>1.5415793829839231</v>
+      </c>
+      <c r="AC40" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD40" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE40" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF40" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG40" t="s">
+        <v>294</v>
+      </c>
+      <c r="AH40" s="14">
+        <v>6.4598243014258108</v>
+      </c>
+      <c r="AI40" s="14">
+        <v>4.8622000714176927</v>
+      </c>
+      <c r="AJ40" s="14">
+        <v>2.9627989223817909E-2</v>
+      </c>
+      <c r="AK40" s="14">
+        <v>1.5679962407843</v>
+      </c>
+    </row>
+    <row r="41" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41" t="s">
+        <v>188</v>
+      </c>
+      <c r="B41" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C41" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D41" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E41" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F41" t="s">
+        <v>294</v>
+      </c>
+      <c r="G41" s="14">
+        <v>5.7763243899059082</v>
+      </c>
+      <c r="H41" s="14">
+        <v>4.2592924944804551</v>
+      </c>
+      <c r="I41" s="14">
+        <v>3.1480166504143182E-2</v>
+      </c>
+      <c r="J41" s="14">
+        <v>1.48555172892131</v>
+      </c>
+      <c r="K41" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L41" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M41" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N41" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O41" t="s">
+        <v>1390</v>
+      </c>
+      <c r="P41" s="14">
+        <v>5.7975068905656606</v>
+      </c>
+      <c r="Q41" s="14">
+        <v>1.327229653624699</v>
+      </c>
+      <c r="R41" s="14">
+        <v>2.0513436235956908</v>
+      </c>
+      <c r="S41" s="14">
+        <v>2.4189336133452701</v>
+      </c>
+      <c r="T41" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U41" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V41" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W41" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X41" t="s">
+        <v>1390</v>
+      </c>
+      <c r="Y41" s="14">
+        <v>5.9165934857162288</v>
+      </c>
+      <c r="Z41" s="14">
+        <v>1.377477853326049</v>
+      </c>
+      <c r="AA41" s="14">
+        <v>2.065218431492966</v>
+      </c>
+      <c r="AB41" s="14">
+        <v>2.473897200897214</v>
+      </c>
+      <c r="AC41" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD41" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE41" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF41" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG41" t="s">
+        <v>1390</v>
+      </c>
+      <c r="AH41" s="14">
+        <v>6.0179815883984684</v>
+      </c>
+      <c r="AI41" s="14">
+        <v>1.4010826296847261</v>
+      </c>
+      <c r="AJ41" s="14">
+        <v>2.1006084881022229</v>
+      </c>
+      <c r="AK41" s="14">
+        <v>2.5162904706115201</v>
+      </c>
+    </row>
+    <row r="42" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42" t="s">
+        <v>188</v>
+      </c>
+      <c r="B42" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C42" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D42" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E42" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F42" t="s">
+        <v>291</v>
+      </c>
+      <c r="G42" s="14">
+        <v>5.0672209833788928</v>
+      </c>
+      <c r="H42" s="14">
+        <v>3.1314576141713042</v>
+      </c>
+      <c r="I42" s="14">
+        <v>3.4356502810493877E-2</v>
+      </c>
+      <c r="J42" s="14">
+        <v>1.901406866397096</v>
+      </c>
+      <c r="K42" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L42" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M42" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N42" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O42" t="s">
+        <v>291</v>
+      </c>
+      <c r="P42" s="14">
+        <v>5.356777286664725</v>
+      </c>
+      <c r="Q42" s="14">
+        <v>3.386290604102062</v>
+      </c>
+      <c r="R42" s="14">
+        <v>3.1576748424325347E-2</v>
+      </c>
+      <c r="S42" s="14">
+        <v>1.938909934138338</v>
+      </c>
+      <c r="T42" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U42" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V42" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W42" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X42" t="s">
+        <v>291</v>
+      </c>
+      <c r="Y42" s="14">
+        <v>5.5379551417973936</v>
+      </c>
+      <c r="Z42" s="14">
+        <v>3.5144937421626299</v>
+      </c>
+      <c r="AA42" s="14">
+        <v>3.1790326156192698E-2</v>
+      </c>
+      <c r="AB42" s="14">
+        <v>1.991671073478571</v>
+      </c>
+      <c r="AC42" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD42" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE42" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF42" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG42" t="s">
+        <v>291</v>
+      </c>
+      <c r="AH42" s="14">
+        <v>5.6328548109941572</v>
+      </c>
+      <c r="AI42" s="14">
+        <v>3.5747189128232</v>
+      </c>
+      <c r="AJ42" s="14">
+        <v>3.2335092474921077E-2</v>
+      </c>
+      <c r="AK42" s="14">
+        <v>2.0258008056960359</v>
+      </c>
+    </row>
+    <row r="43" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43" t="s">
+        <v>188</v>
+      </c>
+      <c r="B43" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C43" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D43" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E43" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F43" t="s">
+        <v>138</v>
+      </c>
+      <c r="G43" s="14">
+        <v>4.7959709172994307</v>
+      </c>
+      <c r="H43" s="14">
+        <v>0.88378390015267205</v>
+      </c>
+      <c r="I43" s="14">
+        <v>1.0286311042222711</v>
+      </c>
+      <c r="J43" s="14">
+        <v>2.883555912924487</v>
+      </c>
+      <c r="K43" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L43" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M43" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N43" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O43" t="s">
+        <v>138</v>
+      </c>
+      <c r="P43" s="14">
+        <v>4.8243396541037162</v>
+      </c>
+      <c r="Q43" s="14">
+        <v>0.9557048141415313</v>
+      </c>
+      <c r="R43" s="14">
+        <v>0.94540546744884868</v>
+      </c>
+      <c r="S43" s="14">
+        <v>2.9232293725133358</v>
+      </c>
+      <c r="T43" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U43" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V43" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W43" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X43" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y43" s="14">
+        <v>4.9432504059780102</v>
+      </c>
+      <c r="Z43" s="14">
+        <v>0.99188728356223399</v>
+      </c>
+      <c r="AA43" s="14">
+        <v>0.95179996864065453</v>
+      </c>
+      <c r="AB43" s="14">
+        <v>2.9995631537751208</v>
+      </c>
+      <c r="AC43" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD43" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE43" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF43" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG43" t="s">
+        <v>138</v>
+      </c>
+      <c r="AH43" s="14">
+        <v>5.027959078452346</v>
+      </c>
+      <c r="AI43" s="14">
+        <v>1.0088844914991659</v>
+      </c>
+      <c r="AJ43" s="14">
+        <v>0.96811023115682437</v>
+      </c>
+      <c r="AK43" s="14">
+        <v>3.0509643557963551</v>
+      </c>
+    </row>
+    <row r="44" spans="1:37" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44" t="s">
+        <v>188</v>
+      </c>
+      <c r="B44" s="14">
+        <v>547.7776417988116</v>
+      </c>
+      <c r="C44" s="14">
+        <v>18.343630242092878</v>
+      </c>
+      <c r="D44" s="14">
+        <v>96.908720553343741</v>
+      </c>
+      <c r="E44" s="14">
+        <v>432.525291003375</v>
+      </c>
+      <c r="F44" t="s">
+        <v>371</v>
+      </c>
+      <c r="G44" s="14">
+        <v>93.393158531176681</v>
+      </c>
+      <c r="H44" s="14">
+        <v>10.76045549875953</v>
+      </c>
+      <c r="I44" s="14">
+        <v>11.130546301407961</v>
+      </c>
+      <c r="J44" s="14">
+        <v>71.502156731009237</v>
+      </c>
+      <c r="K44" s="14">
+        <v>545.92079937631195</v>
+      </c>
+      <c r="L44" s="14">
+        <v>19.83640540201273</v>
+      </c>
+      <c r="M44" s="14">
+        <v>89.067921316529194</v>
+      </c>
+      <c r="N44" s="14">
+        <v>437.01647265777012</v>
+      </c>
+      <c r="O44" t="s">
+        <v>371</v>
+      </c>
+      <c r="P44" s="14">
+        <v>94.753183823713641</v>
+      </c>
+      <c r="Q44" s="14">
+        <v>11.636124080494881</v>
+      </c>
+      <c r="R44" s="14">
+        <v>10.22998360233311</v>
+      </c>
+      <c r="S44" s="14">
+        <v>72.887076140885512</v>
+      </c>
+      <c r="T44" s="14">
+        <v>558.41175182061829</v>
+      </c>
+      <c r="U44" s="14">
+        <v>20.58740102456769</v>
+      </c>
+      <c r="V44" s="14">
+        <v>89.670355878862651</v>
+      </c>
+      <c r="W44" s="14">
+        <v>448.15399491718802</v>
+      </c>
+      <c r="X44" t="s">
+        <v>371</v>
+      </c>
+      <c r="Y44" s="14">
+        <v>97.241560048322768</v>
+      </c>
+      <c r="Z44" s="14">
+        <v>12.076661469747441</v>
+      </c>
+      <c r="AA44" s="14">
+        <v>10.2991768158162</v>
+      </c>
+      <c r="AB44" s="14">
+        <v>74.865721762759122</v>
+      </c>
+      <c r="AC44" s="14">
+        <v>567.98082364704032</v>
+      </c>
+      <c r="AD44" s="14">
+        <v>20.94019144934143</v>
+      </c>
+      <c r="AE44" s="14">
+        <v>91.206967659162885</v>
+      </c>
+      <c r="AF44" s="14">
+        <v>455.83366453853603</v>
+      </c>
+      <c r="AG44" t="s">
+        <v>371</v>
+      </c>
+      <c r="AH44" s="14">
+        <v>98.907913719394216</v>
+      </c>
+      <c r="AI44" s="14">
+        <v>12.283609909945239</v>
+      </c>
+      <c r="AJ44" s="14">
+        <v>10.475665871396149</v>
+      </c>
+      <c r="AK44" s="14">
+        <v>76.148637938052801</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:AK23" xr:uid="{00000000-0001-0000-0600-000000000000}"/>
   <conditionalFormatting sqref="A3:A23">
-    <cfRule type="notContainsBlanks" dxfId="2" priority="1">
+    <cfRule type="notContainsBlanks" dxfId="3" priority="2">
       <formula>LEN(TRIM(A3))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A24:AK44">
+    <cfRule type="notContainsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(A24))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19515,10 +21915,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:L1013">
-    <cfRule type="notContainsBlanks" dxfId="1" priority="1">
+    <cfRule type="notContainsBlanks" dxfId="2" priority="1">
       <formula>LEN(TRIM(A2))&gt;0</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="0" priority="2">
+    <cfRule type="containsBlanks" dxfId="1" priority="2">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19536,6 +21936,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="573d9aa2-0c25-4944-84f7-53a818bcb462">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="785bd73b-6c7f-4235-8928-d0461087983b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5EB07073A11E245877C92B1BAADD97D" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c238704b48ce03d16bf8bb264793b78">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="573d9aa2-0c25-4944-84f7-53a818bcb462" xmlns:ns3="785bd73b-6c7f-4235-8928-d0461087983b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2b09658e3403a73714d8c6b09587f150" ns2:_="" ns3:_="">
     <xsd:import namespace="573d9aa2-0c25-4944-84f7-53a818bcb462"/>
@@ -19736,17 +22147,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="573d9aa2-0c25-4944-84f7-53a818bcb462">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="785bd73b-6c7f-4235-8928-d0461087983b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5B86DD6-4BC3-4212-B9B6-6B2368237363}">
   <ds:schemaRefs>
@@ -19756,6 +22156,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3B5193B-A972-43E7-A9DA-676F799696C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="573d9aa2-0c25-4944-84f7-53a818bcb462"/>
+    <ds:schemaRef ds:uri="785bd73b-6c7f-4235-8928-d0461087983b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E515E57-1109-4EA6-82C5-68CB1C73E5DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19772,15 +22183,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3B5193B-A972-43E7-A9DA-676F799696C8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="573d9aa2-0c25-4944-84f7-53a818bcb462"/>
-    <ds:schemaRef ds:uri="785bd73b-6c7f-4235-8928-d0461087983b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>